<commit_message>
agregando elaboracion de ficha tecnica
</commit_message>
<xml_diff>
--- a/anexo_1.xlsx
+++ b/anexo_1.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yunior\Desktop\proyecto_restaurante\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yunior\Desktop\programa5\costousd\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="51">
   <si>
     <t>ANEXO 1</t>
   </si>
@@ -80,9 +80,6 @@
     <t>PRESENTACIÓN (FOTO) (17)</t>
   </si>
   <si>
-    <t>3% de condimentos</t>
-  </si>
-  <si>
     <t>TOTAL</t>
   </si>
   <si>
@@ -98,9 +95,6 @@
     <t>ÍNDICE DE COSTO TOTAL (21):</t>
   </si>
   <si>
-    <t>ÍNDICE DE COSTO CUC(26):</t>
-  </si>
-  <si>
     <t>REALIZADO POR (23):</t>
   </si>
   <si>
@@ -168,13 +162,29 @@
   </si>
   <si>
     <t>INSTALACIÓN (1):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                                                                                                                                                                                  subtotal</t>
+  </si>
+  <si>
+    <t>PRECIO SIN IMPUESTO</t>
+  </si>
+  <si>
+    <t>IMPUESTO DEL 10%</t>
+  </si>
+  <si>
+    <t>5% de condimentos</t>
+  </si>
+  <si>
+    <t>Observaciones(22)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* &quot;-&quot;??\ _€_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
@@ -654,7 +664,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
@@ -676,6 +685,45 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -702,7 +750,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -748,44 +795,7 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1114,23 +1124,23 @@
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
-      <c r="H3" s="50" t="s">
-        <v>46</v>
-      </c>
-      <c r="I3" s="50"/>
-      <c r="J3" s="50"/>
+      <c r="H3" s="62" t="s">
+        <v>44</v>
+      </c>
+      <c r="I3" s="62"/>
+      <c r="J3" s="62"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B4" s="51" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
+      <c r="B4" s="63" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" s="64"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
+      <c r="F4" s="64"/>
+      <c r="G4" s="64"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="4"/>
@@ -1138,25 +1148,25 @@
       <c r="L4" s="4"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="52"/>
-      <c r="D5" s="52"/>
-      <c r="E5" s="52"/>
+      <c r="C5" s="64"/>
+      <c r="D5" s="64"/>
+      <c r="E5" s="64"/>
       <c r="F5" s="5"/>
       <c r="G5" s="5"/>
-      <c r="H5" s="54" t="s">
+      <c r="H5" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="I5" s="54"/>
-      <c r="J5" s="54"/>
-      <c r="K5" s="54"/>
+      <c r="I5" s="43"/>
+      <c r="J5" s="43"/>
+      <c r="K5" s="43"/>
       <c r="L5" s="6"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B6" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="8"/>
@@ -1165,8 +1175,8 @@
       <c r="G6" s="8"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
-      <c r="J6" s="55"/>
-      <c r="K6" s="55"/>
+      <c r="J6" s="66"/>
+      <c r="K6" s="66"/>
       <c r="L6" s="9"/>
     </row>
     <row r="7" spans="1:12" ht="18.75" x14ac:dyDescent="0.3">
@@ -1199,351 +1209,347 @@
       <c r="L8" s="9"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="56" t="s">
+      <c r="B9" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="58" t="s">
+      <c r="C9" s="69" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="58" t="s">
+      <c r="D9" s="69" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="60" t="s">
+      <c r="E9" s="71" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="61"/>
-      <c r="G9" s="62" t="s">
+      <c r="F9" s="72"/>
+      <c r="G9" s="73" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="64" t="s">
-        <v>35</v>
-      </c>
-      <c r="I9" s="65" t="s">
+      <c r="H9" s="75" t="s">
+        <v>33</v>
+      </c>
+      <c r="I9" s="76" t="s">
         <v>11</v>
       </c>
-      <c r="J9" s="66"/>
+      <c r="J9" s="77"/>
     </row>
     <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="57"/>
-      <c r="C10" s="59"/>
-      <c r="D10" s="59"/>
+      <c r="B10" s="68"/>
+      <c r="C10" s="70"/>
+      <c r="D10" s="70"/>
       <c r="E10" s="14" t="s">
         <v>12</v>
       </c>
       <c r="F10" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="G10" s="63"/>
-      <c r="H10" s="64"/>
-      <c r="I10" s="65" t="s">
+      <c r="G10" s="74"/>
+      <c r="H10" s="75"/>
+      <c r="I10" s="76" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="66"/>
+      <c r="J10" s="77"/>
     </row>
     <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="16"/>
       <c r="B11" s="17">
         <v>1</v>
       </c>
-      <c r="C11" s="36" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="E11" s="39">
+      <c r="C11" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="38">
         <v>0.5</v>
       </c>
-      <c r="F11" s="39">
+      <c r="F11" s="38">
         <v>0</v>
       </c>
-      <c r="G11" s="42">
+      <c r="G11" s="41">
         <v>4.0262000000000002</v>
       </c>
-      <c r="H11" s="38">
+      <c r="H11" s="37">
         <v>2.0133999999999999</v>
       </c>
-      <c r="I11" s="44" t="s">
-        <v>42</v>
-      </c>
-      <c r="J11" s="45"/>
+      <c r="I11" s="56" t="s">
+        <v>40</v>
+      </c>
+      <c r="J11" s="57"/>
     </row>
     <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="16"/>
       <c r="B12" s="20">
         <v>2</v>
       </c>
-      <c r="C12" s="36" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="37" t="s">
+      <c r="C12" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="38">
+      <c r="D12" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="37">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="F12" s="38">
+      <c r="F12" s="37">
         <v>0</v>
       </c>
-      <c r="G12" s="42">
+      <c r="G12" s="41">
         <v>623.95000000000005</v>
       </c>
-      <c r="H12" s="38">
+      <c r="H12" s="37">
         <v>0.312</v>
       </c>
-      <c r="I12" s="46"/>
-      <c r="J12" s="47"/>
+      <c r="I12" s="58"/>
+      <c r="J12" s="59"/>
     </row>
     <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="16"/>
       <c r="B13" s="20">
         <v>3</v>
       </c>
-      <c r="C13" s="40" t="s">
-        <v>31</v>
-      </c>
-      <c r="D13" s="37" t="s">
-        <v>32</v>
-      </c>
-      <c r="E13" s="38">
+      <c r="C13" s="39" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="36" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" s="37">
         <v>0.5</v>
       </c>
-      <c r="F13" s="38">
+      <c r="F13" s="37">
         <v>0</v>
       </c>
-      <c r="G13" s="42">
+      <c r="G13" s="41">
         <v>2.1427</v>
       </c>
-      <c r="H13" s="38">
+      <c r="H13" s="37">
         <v>1.0713999999999999</v>
       </c>
-      <c r="I13" s="46"/>
-      <c r="J13" s="47"/>
+      <c r="I13" s="58"/>
+      <c r="J13" s="59"/>
     </row>
     <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="16"/>
       <c r="B14" s="20">
         <v>4</v>
       </c>
-      <c r="C14" s="40" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="E14" s="38">
+      <c r="C14" s="39" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" s="37">
         <v>0.5</v>
       </c>
-      <c r="F14" s="38">
+      <c r="F14" s="37">
         <v>0</v>
       </c>
-      <c r="G14" s="42">
+      <c r="G14" s="41">
         <v>97</v>
       </c>
-      <c r="H14" s="38">
+      <c r="H14" s="37">
         <v>9.6999999999999993</v>
       </c>
-      <c r="I14" s="48"/>
-      <c r="J14" s="49"/>
+      <c r="I14" s="60"/>
+      <c r="J14" s="61"/>
     </row>
     <row r="15" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="16"/>
       <c r="B15" s="20">
         <v>5</v>
       </c>
-      <c r="C15" s="40" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" s="38">
+      <c r="C15" s="39" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" s="37">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F15" s="38">
+      <c r="F15" s="37">
         <v>0</v>
       </c>
-      <c r="G15" s="42">
+      <c r="G15" s="41">
         <v>27.45</v>
       </c>
-      <c r="H15" s="38">
+      <c r="H15" s="37">
         <v>6.8624999999999998</v>
       </c>
-      <c r="I15" s="67" t="s">
+      <c r="I15" s="54" t="s">
         <v>15</v>
       </c>
-      <c r="J15" s="68"/>
+      <c r="J15" s="55"/>
     </row>
     <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="16"/>
       <c r="B16" s="20">
         <v>6</v>
       </c>
-      <c r="C16" s="40" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="E16" s="38">
+      <c r="C16" s="39" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" s="37">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F16" s="38">
+      <c r="F16" s="37">
         <v>0</v>
       </c>
-      <c r="G16" s="42">
+      <c r="G16" s="41">
         <v>28.48</v>
       </c>
-      <c r="H16" s="38">
+      <c r="H16" s="37">
         <v>7.12</v>
       </c>
-      <c r="I16" s="44" t="s">
-        <v>43</v>
-      </c>
-      <c r="J16" s="45"/>
+      <c r="I16" s="56" t="s">
+        <v>41</v>
+      </c>
+      <c r="J16" s="57"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="16"/>
       <c r="B17" s="17">
         <v>7</v>
       </c>
-      <c r="C17" s="36" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="E17" s="38">
+      <c r="C17" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="37">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="F17" s="39">
+      <c r="F17" s="38">
         <v>0</v>
       </c>
-      <c r="G17" s="42">
+      <c r="G17" s="41">
         <v>180.59559999999999</v>
       </c>
-      <c r="H17" s="38">
+      <c r="H17" s="37">
         <v>0.90300000000000002</v>
       </c>
-      <c r="I17" s="46"/>
-      <c r="J17" s="47"/>
+      <c r="I17" s="58"/>
+      <c r="J17" s="59"/>
     </row>
     <row r="18" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="16"/>
       <c r="B18" s="20">
         <v>8</v>
       </c>
-      <c r="C18" s="40" t="s">
+      <c r="C18" s="39" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="36" t="s">
         <v>37</v>
       </c>
-      <c r="D18" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" s="38">
+      <c r="E18" s="37">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="F18" s="38">
+      <c r="F18" s="37">
         <v>0</v>
       </c>
-      <c r="G18" s="41">
+      <c r="G18" s="40">
         <v>108.7</v>
       </c>
-      <c r="H18" s="38">
+      <c r="H18" s="37">
         <v>0.54349999999999998</v>
       </c>
-      <c r="I18" s="48"/>
-      <c r="J18" s="49"/>
+      <c r="I18" s="60"/>
+      <c r="J18" s="61"/>
     </row>
     <row r="19" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="16"/>
       <c r="B19" s="20">
         <v>9</v>
       </c>
-      <c r="C19" s="40" t="s">
-        <v>40</v>
-      </c>
-      <c r="D19" s="37" t="s">
-        <v>39</v>
-      </c>
-      <c r="E19" s="38">
+      <c r="C19" s="39" t="s">
+        <v>38</v>
+      </c>
+      <c r="D19" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="E19" s="37">
         <v>2E-3</v>
       </c>
-      <c r="F19" s="38">
+      <c r="F19" s="37">
         <v>0</v>
       </c>
-      <c r="G19" s="41">
+      <c r="G19" s="40">
         <v>5.43</v>
       </c>
-      <c r="H19" s="38">
+      <c r="H19" s="37">
         <v>1.09E-2</v>
       </c>
-      <c r="I19" s="67" t="s">
+      <c r="I19" s="54" t="s">
         <v>16</v>
       </c>
-      <c r="J19" s="68"/>
+      <c r="J19" s="55"/>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B20" s="20">
         <v>10</v>
       </c>
-      <c r="C20" s="40" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="E20" s="38">
+      <c r="C20" s="39" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20" s="37">
         <v>1E-3</v>
       </c>
-      <c r="F20" s="38">
+      <c r="F20" s="37">
         <v>0</v>
       </c>
-      <c r="G20" s="41">
+      <c r="G20" s="40">
         <v>180.12</v>
       </c>
-      <c r="H20" s="38">
+      <c r="H20" s="37">
         <v>0.18010000000000001</v>
       </c>
-      <c r="I20" s="44" t="s">
-        <v>44</v>
-      </c>
-      <c r="J20" s="45"/>
+      <c r="I20" s="56" t="s">
+        <v>42</v>
+      </c>
+      <c r="J20" s="57"/>
     </row>
     <row r="21" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="20"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="37"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="38"/>
-      <c r="G21" s="41"/>
-      <c r="H21" s="38">
-        <f>SUM(H11:H20)</f>
-        <v>28.716799999999999</v>
-      </c>
-      <c r="I21" s="48"/>
-      <c r="J21" s="49"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="36"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="37"/>
+      <c r="G21" s="40"/>
+      <c r="I21" s="60"/>
+      <c r="J21" s="61"/>
     </row>
     <row r="22" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B22" s="20"/>
-      <c r="C22" s="40"/>
-      <c r="D22" s="37"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="38"/>
-      <c r="G22" s="41"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="67" t="s">
+      <c r="C22" s="39"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="37"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="37"/>
+      <c r="I22" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="J22" s="68"/>
+      <c r="J22" s="55"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B23" s="20"/>
-      <c r="C23" s="40"/>
-      <c r="D23" s="37"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="38"/>
-      <c r="G23" s="41"/>
-      <c r="H23" s="38"/>
+      <c r="C23" s="39"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="37"/>
+      <c r="G23" s="40"/>
+      <c r="H23" s="37"/>
       <c r="I23" s="18"/>
       <c r="J23" s="19"/>
     </row>
@@ -1553,31 +1559,36 @@
       <c r="D24" s="22"/>
       <c r="E24" s="23"/>
       <c r="F24" s="23"/>
-      <c r="G24" s="43"/>
+      <c r="G24" s="42"/>
       <c r="H24" s="23"/>
       <c r="I24" s="24"/>
       <c r="J24" s="25"/>
     </row>
     <row r="25" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="69"/>
-      <c r="C25" s="70"/>
-      <c r="D25" s="70"/>
-      <c r="E25" s="70"/>
-      <c r="F25" s="70"/>
-      <c r="G25" s="70"/>
-      <c r="H25" s="71"/>
-      <c r="I25" s="23"/>
+      <c r="B25" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="45"/>
+      <c r="D25" s="45"/>
+      <c r="E25" s="45"/>
+      <c r="F25" s="45"/>
+      <c r="G25" s="45"/>
+      <c r="H25" s="46"/>
+      <c r="I25" s="37">
+        <f>SUM(H11:H24)</f>
+        <v>28.716799999999999</v>
+      </c>
       <c r="J25" s="23"/>
       <c r="K25" s="24"/>
       <c r="L25" s="24"/>
     </row>
     <row r="26" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="H26" s="26" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="I26" s="27">
-        <f>3/100*H21</f>
-        <v>0.86150399999999994</v>
+        <f>(5/100*I25)</f>
+        <v>1.43584</v>
       </c>
       <c r="J26" s="27">
         <f>SUM(J12:J25)</f>
@@ -1586,10 +1597,11 @@
     </row>
     <row r="27" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="H27" s="28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I27" s="27">
-        <v>29.578299999999999</v>
+        <f>SUM(I25,I26)</f>
+        <v>30.152639999999998</v>
       </c>
       <c r="J27" s="29">
         <f>J25+J26</f>
@@ -1597,102 +1609,125 @@
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B29" s="72" t="s">
+      <c r="B29" s="47" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="48"/>
+      <c r="D29" s="48"/>
+      <c r="E29" s="27">
+        <f>I27</f>
+        <v>30.152639999999998</v>
+      </c>
+      <c r="H29" s="30" t="s">
         <v>20</v>
-      </c>
-      <c r="C29" s="73"/>
-      <c r="D29" s="73"/>
-      <c r="E29" s="27">
-        <v>29.578299999999999</v>
-      </c>
-      <c r="H29" s="30" t="s">
-        <v>21</v>
       </c>
       <c r="K29" s="30"/>
       <c r="L29" s="30"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B30" s="74" t="s">
+    <row r="30" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="49" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="50"/>
+      <c r="D30" s="50"/>
+      <c r="E30" s="78">
+        <f>ROUNDUP((E32+E31)/5,0)*5</f>
+        <v>265</v>
+      </c>
+      <c r="G30" s="51" t="s">
         <v>22</v>
       </c>
-      <c r="C30" s="75"/>
-      <c r="D30" s="75"/>
-      <c r="E30" s="31">
+      <c r="H30" s="51"/>
+      <c r="I30" s="51"/>
+      <c r="J30" s="31">
+        <f>I27/E30</f>
+        <v>0.11378354716981132</v>
+      </c>
+      <c r="L30" s="32"/>
+    </row>
+    <row r="31" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="49" t="s">
+        <v>48</v>
+      </c>
+      <c r="C31" s="50"/>
+      <c r="D31" s="50"/>
+      <c r="E31" s="78">
+        <f>(10/100*E32)</f>
+        <v>24</v>
+      </c>
+      <c r="G31" s="53"/>
+      <c r="H31" s="53"/>
+      <c r="I31" s="53"/>
+      <c r="L31" s="32"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B32" s="49" t="s">
+        <v>47</v>
+      </c>
+      <c r="C32" s="50"/>
+      <c r="D32" s="50"/>
+      <c r="E32" s="78">
         <v>240</v>
       </c>
-      <c r="G30" s="76" t="s">
-        <v>23</v>
-      </c>
-      <c r="H30" s="76"/>
-      <c r="I30" s="76"/>
-      <c r="J30" s="76"/>
-      <c r="K30" s="32">
-        <f>J27/E30</f>
-        <v>0</v>
-      </c>
-      <c r="L30" s="33"/>
-    </row>
-    <row r="31" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G31" s="78" t="s">
-        <v>24</v>
-      </c>
-      <c r="H31" s="78"/>
-      <c r="I31" s="78"/>
-      <c r="J31" s="32">
-        <f>I27/E30</f>
-        <v>0.12324291666666666</v>
-      </c>
-      <c r="L31" s="33"/>
+      <c r="L32" s="31"/>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="C33" s="9"/>
-      <c r="D33" s="11"/>
+      <c r="B33" s="49"/>
+      <c r="C33" s="50"/>
+      <c r="D33" s="50"/>
       <c r="E33" s="3"/>
       <c r="F33" s="11"/>
-      <c r="G33" s="34"/>
+      <c r="G33" s="33"/>
       <c r="H33" s="11"/>
       <c r="I33" s="9"/>
       <c r="J33" s="9"/>
       <c r="K33" s="9"/>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B34" s="35"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="35"/>
-      <c r="F34" s="35"/>
-      <c r="G34" s="35"/>
-      <c r="H34" s="35"/>
+      <c r="B34" s="34"/>
+      <c r="C34" s="34"/>
+      <c r="D34" s="34"/>
+      <c r="E34" s="34"/>
+      <c r="F34" s="34"/>
+      <c r="G34" s="34"/>
+      <c r="H34" s="34"/>
+    </row>
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B35" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="C35" s="50"/>
+      <c r="D35" s="50"/>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="F36" s="77"/>
-      <c r="G36" s="77"/>
+      <c r="F36" s="52"/>
+      <c r="G36" s="52"/>
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="F37" s="77"/>
-      <c r="G37" s="77"/>
+      <c r="F37" s="52"/>
+      <c r="G37" s="52"/>
     </row>
     <row r="38" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="F38" s="77"/>
-      <c r="G38" s="77"/>
+      <c r="F38" s="52"/>
+      <c r="G38" s="52"/>
     </row>
     <row r="39" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B39" s="54" t="s">
+      <c r="B39" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="C39" s="43"/>
+      <c r="D39" s="43"/>
+      <c r="E39" s="43"/>
+      <c r="F39" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="G39" s="43"/>
+      <c r="H39" s="43"/>
+      <c r="I39" s="43"/>
+      <c r="J39" s="43" t="s">
         <v>25</v>
       </c>
-      <c r="C39" s="54"/>
-      <c r="D39" s="54"/>
-      <c r="E39" s="54"/>
-      <c r="F39" s="54" t="s">
-        <v>26</v>
-      </c>
-      <c r="G39" s="54"/>
-      <c r="H39" s="54"/>
-      <c r="I39" s="54"/>
-      <c r="J39" s="54" t="s">
-        <v>27</v>
-      </c>
-      <c r="K39" s="54"/>
+      <c r="K39" s="43"/>
     </row>
     <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="D40" s="8"/>
@@ -1702,21 +1737,7 @@
       <c r="H40" s="8"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="F39:I39"/>
-    <mergeCell ref="J39:K39"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="F36:G38"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="I15:J15"/>
-    <mergeCell ref="I16:J18"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="I20:J21"/>
-    <mergeCell ref="I22:J22"/>
+  <mergeCells count="32">
     <mergeCell ref="I11:J14"/>
     <mergeCell ref="H3:J3"/>
     <mergeCell ref="B4:G4"/>
@@ -1731,6 +1752,24 @@
     <mergeCell ref="H9:H10"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="I10:J10"/>
+    <mergeCell ref="I15:J15"/>
+    <mergeCell ref="I16:J18"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="I20:J21"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="J39:K39"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="F36:G38"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="G30:I30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>